<commit_message>
Updated Amsh Shrestha timesheets
</commit_message>
<xml_diff>
--- a/AmshShrestha_S394695/Individual Timesheets - Amsh Shrestha(S394695).xlsx
+++ b/AmshShrestha_S394695/Individual Timesheets - Amsh Shrestha(S394695).xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17180" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Individual Timesheets for all s" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Individual Timesheets for all s" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -922,7 +922,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
@@ -1023,134 +1022,131 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Week 08</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>S394695</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Amsh Shrestha</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Planned and implemented Group Dashboard restructuring: added /groups/:id routing, split GroupsPage into list-only view, built GroupDashboardPage with Overview/Transactions/Members tabs</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Week 08</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>S394695</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Amsh Shrestha</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Built AddExpenseModal component (equal/unequal/percentage split as an overlay modal) and wired Transactions tab to merge expense + settlement history</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Week 08</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>S394695</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Amsh Shrestha</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Verified dashboard end-to-end: clean TypeScript build and lint, full API smoke test (all split methods, balances, settlements, rename/remove member), ran client+server locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Week 08</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>S394695</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Amsh Shrestha</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Git hygiene: added bin/obj to .gitignore, untracked SecureVault build artifacts causing spurious diffs on rebuild</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Week 08</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>S394695</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Amsh Shrestha</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Merged amsh branch into main</t>
+        </is>
+      </c>
+    </row>
     <row r="159" ht="13" customHeight="1">
       <c r="D159" s="3" t="n"/>
     </row>

</xml_diff>

<commit_message>
Project documentation and Amsh Shrestha Individual timesheel updates
</commit_message>
<xml_diff>
--- a/AmshShrestha_S394695/Individual Timesheets - Amsh Shrestha(S394695).xlsx
+++ b/AmshShrestha_S394695/Individual Timesheets - Amsh Shrestha(S394695).xlsx
@@ -1297,6 +1297,272 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Week 08</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>S394695</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Amsh Shrestha</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Modernised the UI: added light/dark theme toggle, restyled the header, notification bell and all pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Week 08</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>S394695</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Amsh Shrestha</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Added expense split suggestions: split amounts auto balance in AddExpenseModal, plus a member search endpoint for adding members to a group</t>
+        </is>
+      </c>
+    </row>
+    <row r="46"/>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Week 09</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>S394695</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Amsh Shrestha</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Made split auto balancing work for unequal ($) splits too, suggested values show in italics; added show/hide password button on the sign in page</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Week 09</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>S394695</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Amsh Shrestha</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Fixed Biome lint and formatting issues in the client</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Week 09</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>S394695</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Amsh Shrestha</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Built receipt photo backend: ExpenseReceipts table + migration, upload/view/remove endpoints (only the payer can upload, 5 MB limit, checks the file is really an image), 6 integration tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Week 09</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>S394695</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Amsh Shrestha</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Built receipt photo frontend: attach/replace/remove with preview in AddExpenseModal, photos compressed before upload, receipt viewer on the Transactions tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Week 09</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>S394695</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Amsh Shrestha</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Fixed local errors after the new migration: applied it to our Supabase database and fixed the empty migration history so dotnet ef database update works again</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Week 09</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>S394695</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Amsh Shrestha</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Added auto refresh to the group dashboard (every 20 seconds and when you come back to the tab), fixed old error messages staying on screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Week 09</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>S394695</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Amsh Shrestha</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Updated project documentation: README, data dictionary (receipts table) and my Project Documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Week 09</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>S394695</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Amsh Shrestha</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Updated Trello board and merged amsh branch into main (PR #9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
     <row r="159" ht="13" customHeight="1">
       <c r="D159" s="3" t="n"/>
     </row>

</xml_diff>